<commit_message>
Update debates data - 2026-09-14
</commit_message>
<xml_diff>
--- a/Debats_SEM_Migration.xlsx
+++ b/Debats_SEM_Migration.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -96,25 +96,25 @@
     <t xml:space="preserve">VS</t>
   </si>
   <si>
-    <t xml:space="preserve">"Un dossier électronique de santé (DES) sûr et fiable doit permettre de faire progresser la numérisation du système de santé" : tel est la première phrase du communiqué de notre commission en août dernier au moment de l'adoption de la nouvelle loi fédérale sur le DES. Personne ne conteste la nécessité de numériser un système dans lequel les échanges électroniques d'informations médicales se généralisent. La population est lasse de devoir subir des examens et des traitements à double, parce que l</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Un dossier électronique de santé (DES) sûr et fiable doit permettre de faire progresser la numérisation du système de santé" : tel est la première phrase du communiqué de notre commission en août dernier au moment de l'adoption de la nouvelle loi fédérale sur le DES. Personne ne conteste la nécessité de numériser un système dans lequel les échanges électroniques d'informations médicales se généralisent. La population est lasse de devoir subir des examens et des traitements à double, parce que leur dossier médical n'a pas été transmis ou parfois trop tardivement. Il y a nécessité d'agir, et ce, d'autant plus que le dossier électronique du patient (DEP) est resté nettement en deçà des attentes en matière de diffusion et d'utilisation.
+    <t xml:space="preserve">"Un dossier électronique de santé (DES) sûr et fiable doit permettre de faire progresser la numérisation du système de santé" : telle est la première phrase du communiqué de notre commission en août dernier au moment de l'adoption du projet de nouvelle loi fédérale sur le dossier électronique de santé. Personne ne conteste la nécessité de numériser un système dans lequel les échanges électroniques d'informations médicales se généralisent. La population est lasse de devoir subir des examens et de</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Un dossier électronique de santé (DES) sûr et fiable doit permettre de faire progresser la numérisation du système de santé" : telle est la première phrase du communiqué de notre commission en août dernier au moment de l'adoption du projet de nouvelle loi fédérale sur le dossier électronique de santé. Personne ne conteste la nécessité de numériser un système dans lequel les échanges électroniques d'informations médicales se généralisent. La population est lasse de devoir subir des examens et des traitements à double, parce que leur dossier médical n'a pas été transmis, ou parfois, trop tardivement. Il y a nécessité d'agir, et ce d'autant plus que le dossier électronique du patient (DEP) est resté nettement en deçà des attentes en matière de diffusion et d'utilisation.
 L'objectif majeur reste le même : rendre disponibles les données de santé pertinentes pour améliorer la qualité des soins, renforcer la sécurité des patients et éviter les redondances. C'est le système d'ouverture du dossier qui change pour les patients : il est désormais automatique et gratuit, avec un droit d'opposition, au lieu d'une démarche active. L'idée de base est que désormais chaque personne dispose d'un parcours de santé continu, indépendamment du lieu et du fournisseur de prestations. 
 Quels sont les principaux éléments du projet ? Premièrement, le principe de l'"opt-out" a été retenu. Comme je l'ai déjà dit, l'ouverture du dossier ne se fera plus à la demande, comme avec le DEP actuel, mais de manière automatique, avec le maintien du droit d'opposition et la possibilité de suppression ou de restriction des droits d'accès.
-Deuxièmement, dans le but d'une participation généralisée, il est prévu d'étendre l'obligation d'utilisation du dossier électronique de santé aux fournisseurs de prestations. Actuellement, tous les hôpitaux et les établissements de soins sont déjà tenus de se raccorder au dossier électronique du patient. Désormais, les médecins, les pharmaciens ou les physiothérapeutes, et d'autres prestataires du domaine ambulatoire qui exercent à la charge de l'assurance obligatoire des soins, devront utiliser le dossier électronique de santé et y saisir toutes les données de santé pertinentes pour un traitement médical. Les réticences des professionnels de la santé étaient l'une des principales causes de l'échec du dossier électronique du patient.
-Troisièmement, au lieu de multiples structures décentralisées qui rendaient complexe la mise en oeuvre du dossier électronique du patient, désormais le projet s'appuie sur une infrastructure centralisée. La commission a en effet décidé à l'unanimité que les cantons devraient se mettre d'accord sur une seule communauté nationale. Pour votre information, le regroupement des différentes communautés de référence a progressé et, depuis que la Poste s'est retirée de l'exploitation du dossier électronique du patient, celui-ci s'oriente déjà vers une communauté unique - fort probablement CARA -, dotée d'une infrastructure technique uniforme. La Confédération reste responsable du système d'information.
-Quatrièmement, l'interopérabilité est l'une des conditions clés de la réussite du projet. Le dossier électronique de santé et le Swiss Health Data Space (SwissHDS) utiliseront des normes et des interfaces communes. Pour information, le dossier électronique de santé a pour but de donner à la population un accès à ses données de santé et de garantir une traçabilité de celles-ci sur le long terme ; le SwissHDS, lui, permet aux fournisseurs de prestations d'échanger des données de manière structurée et automatisée - business to business ou B2B. Les deux projets seront développés en parallèle et étroitement coordonnés. Les modifications faites au niveau des systèmes primaires des fournisseurs de prestations pour leur raccordement au dossier électronique de santé pourront ainsi également être utilisées pour la communication B2B dans le SwissHDS.
+Deuxièmement, dans le but d'une participation généralisée, il est prévu d'étendre l'obligation d'utilisation du dossier électronique de santé aux fournisseurs de prestations. Actuellement, tous les hôpitaux et les établissements de soins sont déjà tenus de se raccorder au dossier électronique du patient. Désormais, les médecins, les pharmaciens ou les physiothérapeutes et d'autres prestataires du domaine ambulatoire qui exercent à la charge de l'assurance obligatoire des soins devront utiliser le dossier électronique de santé et y saisir toutes les données de santé pertinentes pour un traitement médical. Les réticences des professionnels de la santé étaient l'une des principales causes de l'échec du dossier électronique du patient.
+Troisièmement, au lieu de multiples structures décentralisées qui rendaient complexe la mise en oeuvre du dossier électronique du patient, désormais le projet s'appuie sur une infrastructure centralisée. La commission a en effet décidé à l'unanimité que les cantons devraient se mettre d'accord sur une seule communauté nationale. Pour votre information, le regroupement des différentes communautés de référence a progressé et, depuis que la Poste s'est retirée de l'exploitation du dossier électronique du patient, celui-ci s'oriente déjà vers une communauté unique - fort probablement Cara -, dotée d'une infrastructure technique uniforme. La Confédération reste responsable du système d'information.
+Quatrièmement, l'interopérabilité est l'une des conditions clés de la réussite du projet. Le dossier électronique de santé et le Swiss Health Data Space (SwissHDS) utiliseront des normes et des interfaces communes. Pour information, le dossier électronique de santé a pour but de donner à la population un accès à ses données de santé et de garantir une traçabilité de ces dernières sur le long terme ; le SwissHDS, lui, permet aux fournisseurs de prestations d'échanger des données de manière structurée et automatisée - business to business ou B2B. Les deux projets seront développés en parallèle et étroitement coordonnés. Les modifications faites sur le plan des systèmes primaires des fournisseurs de prestations pour leur raccordement au dossier électronique de santé pourront ainsi également être utilisées pour la communication B2B dans le SwissHDS.
 Cinquièmement, un financement clarifié est nécessaire. Si c'est la Confédération qui finance la mise en place et le développement de l'infrastructure, ce sont les cantons qui assumeront les coûts d'exploitation courants et garantiront l'exploitation de la communauté sur leur territoire. Dans son corapport, la Commission des finances de notre conseil relève que les estimations transmises sont imprécises et peu transparentes, notamment parce que l'on souhaite éviter tout risque d'impact négatif sur l'appel d'offres. Elle recommande ainsi de rester attentif aux conséquences budgétaires que pourraient entrainer d'éventuelles modifications apportées au projet.
 Une condition décisive pour l'acceptation et la mise en oeuvre du DES, et qui a préoccupé notre commission, est la confiance en la protection des données. La sécurité des données, leur transition ainsi que leur chiffrement ont été soigneusement analysés. Concernant ce dernier, la commission s'est penchée sur la question d'un éventuel chiffrement de bout en bout (E2EE), sur la base d'une étude de l'EPFL réalisée à la demande de l'Office fédéral de la santé publique. Prenant acte du fait qu'aucun autre système public ou national n'utilise un chiffrement E2EE strict, en raison d'insuffisances techniques, la commission estime que cette solution ne doit pas être inscrite dans la loi. Elle propose toutefois à l'unanimité que les exigences en matière de protection et de sécurité des données, ainsi que la nécessité de chiffrer les données, soient explicitement mentionnées dans un nouvel article 5a. De plus, la commission propose, à l'unanimité, de préciser que la Confédération ne peut traiter les données personnelles "que dans la mesure où cela est nécessaire au bon fonctionnement technique du système d'information DES". Il s'agit de l'article 5 alinéa 5.
-Enfin, à l'unanimité, la commission considère qu'il convient de préciser que le code source des logiciels utilisés doit être publié dans la mesure du possible (open source ; art. 5, al. 8) et que des profils d'autorisation adaptables et faciles à comprendre doivent être mis à disposition (art. 11, al. 5bis et 5ter).
-Une seconde condition est essentielle. Elle concerne la transition entre le dossier électronique du patient (DEP) et le dossier électronique de santé (DES). Quatre points critiques ont été abordés.
+Enfin, à l'unanimité, la commission considère qu'il convient de préciser que le code source des logiciels utilisés doit être publié dans la mesure du possible, donc en "open source" - il s'agit de l'article 5 alinéa 8 - et que des profils d'autorisation adaptables et faciles à comprendre doivent être mis à disposition - article 11 alinéas 5bis et 5ter.
+Une seconde condition est essentielle. Elle concerne la transition entre le DEP et le DES. Quatre points critiques ont été abordés.
 Premièrement, la loi fédérale sur le dossier électronique du patient (LDEP) sera maintenue jusqu'à la mise en oeuvre du DES pour éviter que des lacunes menacent l'exploitation, le financement et les services de base.
 Deuxièmement, le retrait de Post Sanela, prévu à la fin de 2026, doit se faire avec la garantie d'une migration ordonnée vers la communauté de référence Cara - ou vers la plateforme qui sera choisie - sans coûts supplémentaires ni pertes de données. Pour rappel, cela concerne près de 80 000 DEP ouverts, et La Poste, en tant qu'entreprise liée à la Confédération, a une responsabilité particulière à cet égard.
 Troisièmement, la capacité de raccordement technique des fournisseurs de prestations et des systèmes primaires existants avec le DES doit être garantie.
-Quatrièmement, la transition doit être accélérée, mais dans le respect des règles de l'OMC et de la loi fédérale sur les marchés publics (LMP), une procédure de gré à gré étant considérée comme risquée. En bref, une transition stable sans perte de données ni d'investissements est prioritaire. Par courrier, la commission a, de ce fait, invité à l'unanimité le Conseil fédéral à s'engager dans ce sens.
-En conclusion, par 16 voix contre 8, la commission vous recommande d'entrer en matière sur le projet. Bien qu'elle soit d'accord avec l'objectif, une minorité critique en particulier l'infrastructure centralisée, qui, selon elle, nécessitera le lancement d'un nouveau projet informatique important et risqué sur le plan fédéral, ainsi que le droit d'opposition prévu. 
-Je reviendrai à la fin des débats apporter des commentaires sur les propositions des minorités.
+Quatrièmement, la transition doit être accélérée, mais dans le respect des règles de l'OMC et de la loi fédérale sur les marchés publics, une procédure de gré à gré étant considérée comme risquée. En bref, une transition stable sans perte de données ni d'investissements est prioritaire. Par courrier, la commission a, de ce fait, invité à l'unanimité le Conseil fédéral à s'engager dans ce sens.
+En conclusion, par 16 voix contre 8, la commission vous recommande d'entrer en matière sur le projet. Bien qu'elle soit d'accord avec l'objectif, une minorité critique en particulier l'infrastructure centralisée, qui, selon elle, nécessitera le lancement d'un nouveau projet informatique important et risqué sur le plan fédéral, ainsi que le droit d'opposition prévu.
+Je reviendrai à la fin des débats apporter des commentaires sur les propositions de minorités.
 </t>
   </si>
   <si>
@@ -131,6 +131,30 @@
 Der für 2026 vorgesehene Rückzug der Post Sanela Health AG muss so erfolgen, das ist die Meinung der Kommission, dass eine geordnete Migration zu Cara gewährleistet ist. Ich kann Ihnen sagen: 80 000 Dossier sind derzeit bei der Post Sanela Health AG. Da braucht es Lösungen. Die Nachricht, dass die Post aussteigen wird, erreichte die Kommission mitten in der Beratung des Geschäftes. Wir liessen deshalb einen Zusatzbericht anfertigen. Dieser ist aber noch nicht eingetroffen - das war aber auch so geplant. Deshalb bittet Ihre Kommission den Ständerat, sich der Thematik des Anbieters nochmals anzunehmen. Der Ausstieg der Post aus dem EPD könnte auch Auswirkungen auf die Frage der Notwendigkeit einer neuen Ausschreibung haben, was schlussendlich auch zeitliche Konsequenzen haben würde. 
 Die Mehrheit Ihrer Kommission beantragt Ihnen mit 17 zu 8 Stimmen, auf die Vorlage einzutreten. Die Kommissionsmehrheit möchte Ihnen, und wahrscheinlich auch der Bevölkerung, ein Angebot machen, welches ein neues Dossier ermöglicht, das die Schwachstellen des EPD eliminiert. Es ist ein Dossier, wo die Patientinnen und Patienten selbst entscheiden können, wer darauf Zugriff hat, eines, das zentraler gesteuert ist, eines, das nicht die gleichen Fehler wiederholt, die beim EPD gemacht worden sind.
 Ich werde am Schluss noch auf die Minderheiten und den Einzelantrag eingehen. Ich überlasse jetzt gerne das Wort meinem Kommissionssprecher-Kollegen und hoffe, dass Sie ihn verstehen, weil mich haben Sie wahrscheinlich nicht verstanden.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">418690</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baume-Schneider Elisabeth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La motion vise à permettre aux personnes en procédure d'asile, aux bénéficiaires de l'aide sociale ou de prestations complémentaires d'être, en règle générale, tenues de choisir un modèle particulier d'assurance. La motion vise certes à déroger à la règle dans des cas exceptionnels.
+Il convient de préciser que, pour les requérants d'asile et pour les personnes à protéger sans autorisation de séjour, la Confédération et les cantons peuvent d'ores et déjà restreindre le choix de l'assureur, prescr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La motion vise à permettre aux personnes en procédure d'asile, aux bénéficiaires de l'aide sociale ou de prestations complémentaires d'être, en règle générale, tenues de choisir un modèle particulier d'assurance. La motion vise certes à déroger à la règle dans des cas exceptionnels.
+Il convient de préciser que, pour les requérants d'asile et pour les personnes à protéger sans autorisation de séjour, la Confédération et les cantons peuvent d'ores et déjà restreindre le choix de l'assureur, prescrire une forme particulière d'assurance et limiter le choix des fournisseurs de prestations. Cela permet de gérer l'accès au système de santé et d'utiliser les fonds publics de manière économique en garantissant des prix moins élevés. La charge administrative est aussi fortement réduite lorsque les soins de santé des requérants d'asile sont gérés par un seul assureur ou par un petit nombre d'assureurs.
+Les cantons peuvent également accorder une réduction de primes aux assurés dont la condition économique est modeste. Les cantons déterminent à la fois les bénéficiaires et le montant, et peuvent fixer une prime de référence fondée, elle aussi, sur une assurance avec choix limité des fournisseurs de prestations. Il ne s'agit donc pas d'aborder la question de la réduction des primes, mais celle de la prime de référence, qui est basée sur une assurance avec choix limité. Pour le calcul des prestations complémentaires, la prime effective est prise en compte, mais au maximum à hauteur de la prime moyenne cantonale ou régionale. Les bénéficiaires de prestations complémentaires sont dès lors incités à choisir une prime appropriée.
+En résumé, les cantons sont largement compétents en matière de réduction des primes, de prestations complémentaires, d'aide sociale et d'impôts. Ils peuvent donc coordonner ces domaines de manière optimale. La Confédération n'est pas habilitée à édicter des prescriptions allant au-delà de ses propres compétences.
+Dès lors, je vous propose de rejeter la motion.
 </t>
   </si>
   <si>
@@ -183,16 +207,13 @@
     <t xml:space="preserve">NE</t>
   </si>
   <si>
-    <t xml:space="preserve">FR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Conseil national a rejeté cet accord le 17 juin dernier, pas par accident ou par distraction, mais au terme d'un long débat et après avoir refusé une à une toutes les garanties qui auraient pu rendre ce texte un minimum acceptable. Notre commission nous propose aujourd'hui de faire la même chose, à quelques exceptions près. Elle nous propose nouvellement 517 millions de francs pour l'agriculture et un suivi régulier des engagements internationaux ; de l'argent et de la surveillance, là où il </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Conseil national a rejeté cet accord le 17 juin dernier, pas par accident ou par distraction, mais au terme d'un long débat et après avoir refusé une à une toutes les garanties qui auraient pu rendre ce texte un minimum acceptable. Notre commission nous propose aujourd'hui de faire la même chose, à quelques exceptions près. Elle nous propose nouvellement 517 millions de francs pour l'agriculture et un suivi régulier des engagements internationaux ; de l'argent et de la surveillance, là où il aurait fallu des règles strictes et qui fonctionnent. 
-Le premier point sur lequel je veux revenir est la déforestation et le climat. Le Conseil national a refusé de reprendre dans cet accord le Règlement européen sur la déforestation ; un texte qui interdit simplement la commercialisation de produits issus de la destruction des forêts. La commission du Conseil des États n'a malheureusement pas corrigé ce problème. Les chiffres sont pourtant sur la table : l'entrée en vigueur du traité pourrait entraîner la destruction de 900 kilomètres carrés de forêts supplémentaires ; l'équivalent à peu près du canton de Neuchâtel. Nos échanges agricoles avec les pays du Mercosur génèrent aujourd'hui plus de 300 000 tonnes de CO2 par an. L'accord y ajoute à peu près la même chose, c'est-à-dire un doublement. À l'importation, cette hausse tient pour l'essentiel aux dérivés du soja et à la viande bovine. Le projet du Conseil fédéral ne prévoit malheureusement rien pour en réduire l'impact. Rappelons-le : l'élevage bovin est l'un des tout premiers moteurs de la déforestation. Cet accord augmente donc la pression sur la forêt amazonienne et - j'y reviendrai - sur notre agriculture. La déforestation ne concerne pas seulement des tonnes de CO2, mais aussi la destruction d'une biodiversité infiniment précieuse. C'est l'expulsion de peuples autochtones de leurs terres. Ces choses ne se compensent pas. Un suivi ne leur rendra pas leurs terres. 
+    <t xml:space="preserve">Le Conseil national a rejeté cet accord le 17 juin dernier, pas par accident ou par distraction, mais au terme d'un long débat, et après avoir refusé une à une toutes les garanties qui auraient pu rendre ce texte un minimum acceptable. Notre commission nous propose aujourd'hui de faire la même chose, à quelques exceptions près. Elle nous propose nouvellement 517 millions de francs pour l'agriculture et un suivi régulier des engagements internationaux ; de l'argent et de la surveillance là où il </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Conseil national a rejeté cet accord le 17 juin dernier, pas par accident ou par distraction, mais au terme d'un long débat, et après avoir refusé une à une toutes les garanties qui auraient pu rendre ce texte un minimum acceptable. Notre commission nous propose aujourd'hui de faire la même chose, à quelques exceptions près. Elle nous propose nouvellement 517 millions de francs pour l'agriculture et un suivi régulier des engagements internationaux ; de l'argent et de la surveillance là où il aurait fallu des règles strictes et qui fonctionnent.
+Le premier point sur lequel je veux revenir est la déforestation et le climat. Le Conseil national a refusé de reprendre dans cet accord le Règlement européen sur la déforestation ; un texte qui interdit simplement la commercialisation de produits issus de la destruction des forêts. La commission du Conseil des États n'a malheureusement pas corrigé ce problème. Les chiffres sont pourtant sur la table : l'entrée en vigueur du traité pourrait entraîner la destruction de 900 kilomètres carrés de forêts supplémentaires, ce qui équivaut à peu près au canton de Neuchâtel. Nos échanges agricoles avec les pays du Mercosur génèrent aujourd'hui plus de 300 000 tonnes de CO2 par an. L'accord y ajoute à peu près la même chose, c'est-à-dire qu'il y aurait un doublement de ces émissions. À l'importation, cette hausse tient pour l'essentiel aux dérivés du soja et à la viande bovine. Le projet du Conseil fédéral ne prévoit malheureusement rien pour en réduire l'impact. Rappelons-le : l'élevage bovin est l'un des tout premiers moteurs de la déforestation. Cet accord augmente donc la pression sur la forêt amazonienne et - j'y reviendrai - sur notre agriculture. La déforestation ne représente pas seulement des tonnes de CO2, mais aussi la destruction d'une biodiversité infiniment précieuse et l'expulsion de peuples autochtones de leurs terres. Ces choses ne se compensent pas. Un suivi ne leur rendra pas leurs terres.
 Le deuxième point sur lequel je veux revenir est le travail forcé. La gauche a proposé d'interdire l'importation de marchandises produites au moyen du travail forcé. La commission a malheureusement écarté cette proposition et propose, à la place, comme toujours, un suivi. Or, les observateurs de terrain sont clairs : l'esclavage moderne est une réalité bien présente, par exemple dans les plantations de l'agrobusiness. Sur ce plan également, un suivi ne libère personne.
-Concernant ces deux volets, déforestation et travail forcé, cette chambre doit faire ce que l'Europe a fait, poser des règles contraignantes.
+Concernant ces deux volets, déforestation et travail forcé, cette chambre doit faire ce que l'Europe a fait : poser des règles contraignantes.
 Un troisième point important concerne notre agriculture. Nous devrions empêcher l'entrée de produits qui ne respectent pas nos normes, afin que nos agricultrices et agriculteurs puissent vivre dignement de leur travail. Cet accord fait exactement l'inverse. Aucune aide, aussi généreuse soit-elle, ne rendra un producteur suisse concurrentiel face au poulet brésilien. On ne corrige pas une distorsion structurelle avec un crédit d'engagement. Il faut d'ailleurs voir ce traité pour ce qu'il est, un maillon d'une chaîne. La Chine, l'Indonésie, l'Inde, le Chili, demain peut-être la Malaisie : c'est l'accumulation de ces accords qui décidera du sort de l'agriculture et, à moyen terme, de celles et ceux qui veulent produire une alimentation saine et respectueuse de l'environnement.
 J'ajoute un mot sur le contenu exact de ce que nous approuvons. L'accord ouvre un contingent de 1000 tonnes de volaille, 3000 tonnes de viande bovine et 5000 hectolitres de vin en provenance du Mercosur. Ces volumes ne se substituent pas - cela a été dit par le rapporteur - aux concessions existantes. Ils s'ajoutent aux contingents que la Suisse accorde déjà aujourd'hui dans le cadre de l'OMC. Ce point mérite d'être relevé parce que la communication du Conseil fédéral pendant les négociations allait précisément dans l'autre sens. Le Parlement se prononce donc aujourd'hui sur une ouverture plus large que celle qui lui avait été initialement présentée. C'est un problème de méthode autant que de fond.
 Le Conseil national a eu le courage de dire non. Je vous invite à en faire de même et à ne pas entrer en matière.
@@ -244,8 +265,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I6" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I7" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I7"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -667,7 +688,7 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
         <v>28</v>
@@ -677,18 +698,18 @@
         <v>29</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
@@ -697,22 +718,49 @@
         <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" t="s">
         <v>34</v>
       </c>
+      <c r="E6"/>
       <c r="F6" t="s">
         <v>35</v>
       </c>
       <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
         <v>36</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>37</v>
       </c>
-      <c r="I6" t="s">
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
         <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" t="s">
+        <v>30</v>
+      </c>
+      <c r="H7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I7" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update debates data - 2026-09-26
</commit_message>
<xml_diff>
--- a/Debats_SEM_Migration.xlsx
+++ b/Debats_SEM_Migration.xlsx
@@ -236,10 +236,10 @@
     <t xml:space="preserve">ZH</t>
   </si>
   <si>
-    <t xml:space="preserve">Selbstverständlich weiss ich das, Frau Wyss. Ich weiss aber auch, dass wir für die Entwicklungshilfe jährlich 3 Milliarden Franken ausgeben, und für das Asyl- und Flüchtlingswesen geben wir weitere 4 Milliarden Franken aus. Nehmen wir einmal die berühmte Apothekerwaage und legen wir in die eine Schale irgendwelche Programme für die Entwicklungshilfe und in die andere Schale Projekte für die Sicherheit unseres Landes, vor allem für die Sicherheit der kritischen Infrastruktur. Dann wird man sehen,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Selbstverständlich weiss ich das, Frau Wyss. Ich weiss aber auch, dass wir für die Entwicklungshilfe jährlich 3 Milliarden Franken ausgeben, und für das Asyl- und Flüchtlingswesen geben wir weitere 4 Milliarden Franken aus. Nehmen wir einmal die berühmte Apothekerwaage und legen wir in die eine Schale irgendwelche Programme für die Entwicklungshilfe und in die andere Schale Projekte für die Sicherheit unseres Landes, vor allem für die Sicherheit der kritischen Infrastruktur. Dann wird man sehen, dass die zweite Schale viel gewichtiger ist und damit also der Sicherheit viel mehr Gewicht zukommt; die Bevölkerung wird mir recht geben.
+    <t xml:space="preserve">Selbstverständlich weiss ich das, Frau Wyss. Ich weiss aber auch, dass wir für die Entwicklungshilfe jährlich 3 Milliarden Franken ausgeben, und für das Asyl- und Flüchtlingswesen geben wir weitere 4 Milliarden Franken aus. Nehmen wir einmal die berühmte Apothekerwaage, und legen wir in die eine Schale irgendwelche Programme für die Entwicklungshilfe und in die andere Schale Projekte für die Sicherheit unseres Landes, vor allem für die Sicherheit der kritischen Infrastruktur. Dann wird man sehen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selbstverständlich weiss ich das, Frau Wyss. Ich weiss aber auch, dass wir für die Entwicklungshilfe jährlich 3 Milliarden Franken ausgeben, und für das Asyl- und Flüchtlingswesen geben wir weitere 4 Milliarden Franken aus. Nehmen wir einmal die berühmte Apothekerwaage, und legen wir in die eine Schale irgendwelche Programme für die Entwicklungshilfe und in die andere Schale Projekte für die Sicherheit unseres Landes, vor allem für die Sicherheit der kritischen Infrastruktur. Dann wird man sehen, dass die zweite Schale viel gewichtiger ist und damit also der Sicherheit viel mehr Gewicht zukommt; die Bevölkerung wird mir recht geben.
 </t>
   </si>
   <si>

</xml_diff>